<commit_message>
Replace RSCM/R-SCM with RM in C219B test plan
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Psv94Pctv55DFrdiEfWhEP
</commit_message>
<xml_diff>
--- a/C219B_L10_L11_TestPlan_PV_1A00_added.xlsx
+++ b/C219B_L10_L11_TestPlan_PV_1A00_added.xlsx
@@ -1883,6 +1883,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="29" t="n"/>
       <c r="B6" s="28" t="n"/>
@@ -1992,7 +1993,7 @@
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Update BIOS/BMC FW files by RSCM</t>
+          <t>Update BIOS/BMC FW files by RM</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
@@ -2160,7 +2161,7 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Multi-stage, stateful check keyed on the presence of /vol/data/persistent/tests/golden_status.txt on the BMC. If the log doesn't exist yet, the function uploads SoCFPGAGoldenTestSvc.service and fpga_golden_check.py to the BMC, switches GP into golden boot mode (cerberus_utility fpgasetbootmode 0), forces an AC cycle (RSCM rscm_system_ac on M5, gs_pdb_ac_cycle otherwise) to make the mode take effect, and then returns 1 — meaning the first pass of this item after an image/config change always intentionally fails and needs a subsequent PRETEST re-run to actually validate the version. On version mismatch with fpga_gp_fw_upgrade TRUE, it calls _gp_fpga_softnic_upgrade() and then re-generates the golden log (also returning 1) rather than re-checking in the same pass.</t>
+          <t>Multi-stage, stateful check keyed on the presence of /vol/data/persistent/tests/golden_status.txt on the BMC. If the log doesn't exist yet, the function uploads SoCFPGAGoldenTestSvc.service and fpga_golden_check.py to the BMC, switches GP into golden boot mode (cerberus_utility fpgasetbootmode 0), forces an AC cycle (RM rm_system_ac on M5, gs_pdb_ac_cycle otherwise) to make the mode take effect, and then returns 1 — meaning the first pass of this item after an image/config change always intentionally fails and needs a subsequent PRETEST re-run to actually validate the version. On version mismatch with fpga_gp_fw_upgrade TRUE, it calls _gp_fpga_softnic_upgrade() and then re-generates the golden log (also returning 1) rather than re-checking in the same pass.</t>
         </is>
       </c>
     </row>
@@ -2678,7 +2679,7 @@
       <c r="E26" s="74" t="inlineStr">
         <is>
           <t>Two very different code paths: 
-- for prj_stage == "M5" it SFTP-uploads the three HWKEY .bin files to the BMC, then uses a shell command list over usb0 (10.235.100.0/31 point-to-point link) with scp -P 2200 to pull each key onto the GlacierPeak SoC and run cerberus_utility importsignedcert locally there — all three fuse commands (root CA idx 1, intermediate idx 2, device ID idx 0) run under a single rscm_lock.
+- for prj_stage == "M5" it SFTP-uploads the three HWKEY .bin files to the BMC, then uses a shell command list over usb0 (10.235.100.0/31 point-to-point link) with scp -P 2200 to pull each key onto the GlacierPeak SoC and run cerberus_utility importsignedcert locally there — all three fuse commands (root CA idx 1, intermediate idx 2, device ID idx 0) run under a single rm_lock.
 - For other stages it uses a raw pxssh session direct to the GlacierPeak SoC on port 8295 (user admin/admin), with up to 2 retries and a 90s backoff between attempts if the SoC is "busy". HWKey files are deleted from the BMC after fusing in both paths.</t>
         </is>
       </c>
@@ -2708,7 +2709,7 @@
           <t>- Security/identity-relevant, one-time step, M3-only. 
 - Unlike the Manticore/TIP flow this checks each slot independently — a partially-provisioned board (e.g. slot0 done, slot1 not) only provisions the missing slot. 
 - No verification of the -setCertificate output content is performed. 
-- Uses self.rscm_lock("RSCM", ...) around the actual burn to avoid concurrent RSCM access from other test threads.
+- Uses self.rm_lock("RM", ...) around the actual burn to avoid concurrent RM access from other test threads.
 - After both slots are set, it resets the FPGA and sleeps 300s before the final confirmation check.</t>
         </is>
       </c>
@@ -3125,13 +3126,13 @@
       </c>
       <c r="D45" s="11" t="inlineStr">
         <is>
-          <t>PASS if 5/5 pings succeed (or the RSCM-routed SSH connect succeeds).</t>
+          <t>PASS if 5/5 pings succeed (or the RM-routed SSH connect succeeds).</t>
         </is>
       </c>
       <c r="E45" s="11" t="inlineStr">
         <is>
           <t>M1/M3: via a direct ICMP ping
-M5: ping via an SSH-through-RSCM reachability check</t>
+M5: ping via an SSH-through-RM reachability check</t>
         </is>
       </c>
     </row>
@@ -3369,7 +3370,7 @@
       </c>
       <c r="C55" s="13" t="inlineStr">
         <is>
-          <t>Runs fpgadiagnostics -dumpHealth (via a stage-appropriate SSH route: direct M3, RSCM-jumper M3, or RSCM-serial-proxy M5) and parses per-subsystem [FPGA-XXX] health lines, with specific waivers for known FPGA-NETWORK and FPGA-CONFIG warnings, and a one-time auto-reboot self-heal if the PCIe link status reads "WARNING" while in App mode.</t>
+          <t>Runs fpgadiagnostics -dumpHealth (via a stage-appropriate SSH route: direct M3, RM-jumper M3, or RM-serial-proxy M5) and parses per-subsystem [FPGA-XXX] health lines, with specific waivers for known FPGA-NETWORK and FPGA-CONFIG warnings, and a one-time auto-reboot self-heal if the PCIe link status reads "WARNING" while in App mode.</t>
         </is>
       </c>
       <c r="D55" s="13" t="inlineStr">
@@ -4172,7 +4173,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Security/identity-relevant, one-time step, M3-only. Unlike the Manticore/TIP flow this checks each slot independently — a partially-provisioned board (e.g. slot0 done, slot1 not) only provisions the missing slot. No verification of the -setCertificate output content is performed ("Aligned with T6F, based on MTE/Casper approval, no check is required in set Cert" — the old response-code check is commented out). Uses self.rscm_lock("RSCM", ...) around the actual burn to avoid concurrent RSCM access from other test threads. After both slots are set, it resets the FPGA (gp_fpga_reset via cerberus_utility) and sleeps 300s before the final confirmation check.</t>
+          <t>Security/identity-relevant, one-time step, M3-only. Unlike the Manticore/TIP flow this checks each slot independently — a partially-provisioned board (e.g. slot0 done, slot1 not) only provisions the missing slot. No verification of the -setCertificate output content is performed ("Aligned with T6F, based on MTE/Casper approval, no check is required in set Cert" — the old response-code check is commented out). Uses self.rm_lock("RM", ...) around the actual burn to avoid concurrent RM access from other test threads. After both slots are set, it resets the FPGA (gp_fpga_reset via cerberus_utility) and sleeps 300s before the final confirmation check.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -4203,7 +4204,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Security/identity-relevant, one-time step. Migrated/renamed from pcie.py (per docstring, 20260422). Docstring explicitly calls out a fix for error 0x2904: "modified the provisioning order to ensure the root CA is written before the Device ID". Two very different code paths: for prj_stage == "M5" it SFTP-uploads the three HWKEY .bin files to the BMC, then uses a shell command list over usb0 (10.235.100.0/31 point-to-point link) with scp -P 2200 to pull each key onto the GlacierPeak SoC and run cerberus_utility importsignedcert locally there — all three fuse commands (root CA idx 1, intermediate idx 2, device ID idx 0) run under a single rscm_lock. For other stages it uses a raw pxssh session direct to the GlacierPeak SoC on port 8295 (user admin/admin), with up to 2 retries and a 90s backoff between attempts if the SoC is "busy". HWKey files are deleted from the BMC after fusing in both paths.</t>
+          <t>Security/identity-relevant, one-time step. Migrated/renamed from pcie.py (per docstring, 20260422). Docstring explicitly calls out a fix for error 0x2904: "modified the provisioning order to ensure the root CA is written before the Device ID". Two very different code paths: for prj_stage == "M5" it SFTP-uploads the three HWKEY .bin files to the BMC, then uses a shell command list over usb0 (10.235.100.0/31 point-to-point link) with scp -P 2200 to pull each key onto the GlacierPeak SoC and run cerberus_utility importsignedcert locally there — all three fuse commands (root CA idx 1, intermediate idx 2, device ID idx 0) run under a single rm_lock. For other stages it uses a raw pxssh session direct to the GlacierPeak SoC on port 8295 (user admin/admin), with up to 2 retries and a 90s backoff between attempts if the SoC is "busy". HWKey files are deleted from the BMC after fusing in both paths.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -4540,7 +4541,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>"For SKU1 and L11 only" per docstring. SN-format heuristic: a 13-character alphanumeric string is treated as already-correct; anything else is assumed hex-encoded and is bytes.fromhex().decode('ascii')-converted. If conversion fails or the format is still wrong, it uploads rtx-pro-6000-fru-repair_v4.sh and rtx-pro-6000-fru-write_v1.sh to the BMC and runs a repair pipeline (read raw FRU → hexdump → repair script → write script) under an rscm_lock, for cassette 8 (102) and cassette 10 (106) targets.</t>
+          <t>"For SKU1 and L11 only" per docstring. SN-format heuristic: a 13-character alphanumeric string is treated as already-correct; anything else is assumed hex-encoded and is bytes.fromhex().decode('ascii')-converted. If conversion fails or the format is still wrong, it uploads rtx-pro-6000-fru-repair_v4.sh and rtx-pro-6000-fru-write_v1.sh to the BMC and runs a repair pipeline (read raw FRU → hexdump → repair script → write script) under an rm_lock, for cassette 8 (102) and cassette 10 (106) targets.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -5062,13 +5063,13 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>PASS if 5/5 pings succeed (or the RSCM-routed SSH connect succeeds).</t>
+          <t>PASS if 5/5 pings succeed (or the RM-routed SSH connect succeeds).</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
           <t>M1/M3: via a direct ICMP ping
-M5: ping via an SSH-through-RSCM reachability check</t>
+M5: ping via an SSH-through-RM reachability check</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -5612,7 +5613,7 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Runs fpgadiagnostics -dumpHealth (via a stage-appropriate SSH route: direct M3, RSCM-jumper M3, or RSCM-serial-proxy M5) and parses per-subsystem [FPGA-XXX] health lines, with specific waivers for known FPGA-NETWORK and FPGA-CONFIG warnings, and a one-time auto-reboot self-heal if the PCIe link status reads "WARNING" while in App mode.</t>
+          <t>Runs fpgadiagnostics -dumpHealth (via a stage-appropriate SSH route: direct M3, RM-jumper M3, or RM-serial-proxy M5) and parses per-subsystem [FPGA-XXX] health lines, with specific waivers for known FPGA-NETWORK and FPGA-CONFIG warnings, and a one-time auto-reboot self-heal if the PCIe link status reads "WARNING" while in App mode.</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -6327,7 +6328,7 @@
     <col width="9.140625" customWidth="1" style="21" min="14" max="14"/>
     <col width="9.140625" customWidth="1" style="21" min="15" max="15"/>
     <col width="9.140625" customWidth="1" style="22" min="16" max="16"/>
-    <col hidden="1" style="80" min="17" max="25"/>
+    <col hidden="1" width="13" customWidth="1" style="80" min="17" max="25"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customFormat="1" customHeight="1" s="1">
@@ -6577,7 +6578,7 @@
       </c>
       <c r="C7" s="43" t="inlineStr">
         <is>
-          <t>Check RSCM firmware and configuration versions (Cerberus, PCD ID, PFM ID, AM64 stack, CPLD). Auto-update if mismatch and upgrade is allowed.</t>
+          <t>Check RM firmware and configuration versions (Cerberus, PCD ID, PFM ID, AM64 stack, CPLD). Auto-update if mismatch and upgrade is allowed.</t>
         </is>
       </c>
       <c r="D7" s="40" t="inlineStr">
@@ -6613,7 +6614,7 @@
       </c>
       <c r="C8" s="82" t="inlineStr">
         <is>
-          <t>Check RSCM Health Status</t>
+          <t>Check RM Health Status</t>
         </is>
       </c>
       <c r="D8" s="83" t="inlineStr">
@@ -6652,7 +6653,7 @@
       <c r="C9" s="82" t="inlineStr">
         <is>
           <t>Check POWERSHELF Product Name
-Check RSCM Manager Type</t>
+Check RM Manager Type</t>
         </is>
       </c>
       <c r="D9" s="83" t="n"/>
@@ -6684,12 +6685,12 @@
       </c>
       <c r="C10" s="43" t="inlineStr">
         <is>
-          <t>Checks UUT system information via the R-SCM interface and compares it with the expected configuration values .</t>
+          <t>Checks UUT system information via the RM interface and compares it with the expected configuration values .</t>
         </is>
       </c>
       <c r="D10" s="40" t="inlineStr">
         <is>
-          <t>Pass All fields (MAC, SN, BIOS version, BMC version, CPLD versions, CPU count, and memory size) match expected values. Or mismatched fields are successfully auto-updated (if allowed). Fail Unable to retrieve system info from R-SCM. Mismatched field(s) and auto-upgrade is either disabled or unsuccessful.</t>
+          <t>Pass All fields (MAC, SN, BIOS version, BMC version, CPLD versions, CPU count, and memory size) match expected values. Or mismatched fields are successfully auto-updated (if allowed). Fail Unable to retrieve system info from RM. Mismatched field(s) and auto-upgrade is either disabled or unsuccessful.</t>
         </is>
       </c>
       <c r="E10" s="40" t="n"/>
@@ -6762,7 +6763,7 @@
       </c>
       <c r="E12" s="40" t="inlineStr">
         <is>
-          <t>Multi-stage, stateful check keyed on the presence of /vol/data/persistent/tests/golden_status.txt on the BMC. If the log doesn't exist yet, the function uploads SoCFPGAGoldenTestSvc.service and fpga_golden_check.py to the BMC, switches GP into golden boot mode (cerberus_utility fpgasetbootmode 0), forces an AC cycle (RSCM rscm_system_ac on M5, gs_pdb_ac_cycle otherwise) to make the mode take effect, and then returns 1 — meaning the first pass of this item after an image/config change always intentionally fails and needs a subsequent PRETEST re-run to actually validate the version. On version mismatch with fpga_gp_fw_upgrade TRUE, it calls _gp_fpga_softnic_upgrade() and then re-generates the golden log (also returning 1) rather than re-checking in the same pass.</t>
+          <t>Multi-stage, stateful check keyed on the presence of /vol/data/persistent/tests/golden_status.txt on the BMC. If the log doesn't exist yet, the function uploads SoCFPGAGoldenTestSvc.service and fpga_golden_check.py to the BMC, switches GP into golden boot mode (cerberus_utility fpgasetbootmode 0), forces an AC cycle (RM rm_system_ac on M5, gs_pdb_ac_cycle otherwise) to make the mode take effect, and then returns 1 — meaning the first pass of this item after an image/config change always intentionally fails and needs a subsequent PRETEST re-run to actually validate the version. On version mismatch with fpga_gp_fw_upgrade TRUE, it calls _gp_fpga_softnic_upgrade() and then re-generates the golden log (also returning 1) rather than re-checking in the same pass.</t>
         </is>
       </c>
       <c r="F12" s="75" t="n"/>
@@ -7244,7 +7245,7 @@
       </c>
       <c r="C26" s="82" t="inlineStr">
         <is>
-          <t>Check the PSU firmware version on the power shelf via R-SCM for the current UUT. This function only performs the check on master nodes.</t>
+          <t>Check the PSU firmware version on the power shelf via RM for the current UUT. This function only performs the check on master nodes.</t>
         </is>
       </c>
       <c r="D26" s="83" t="inlineStr">
@@ -7253,7 +7254,7 @@
 - UUT is a master node.
 - All PSU serial numbers, manufacturers, and firmware versions match expected values.
 - Fail
-- Unable to get R-SCM IP.
+- Unable to get RM IP.
 - PSU information cannot be retrieved or parsed.
 - PSU not found in the expected list.
 - Firmware version mismatch and auto-upgrade fails.</t>
@@ -7280,12 +7281,12 @@
 -        Completion Code
 - - - - -  If mismatch - - - - -
 [Upgrade PSU firmware version]
-Check fw package exists in RSCM:
+Check fw package exists in RM:
 -        show manager tftp list
 Upload fw to Rack-SCM
 -        set manager tftp get -s {IP} -f {FILE}
 Fw Upgrade
--       rscm_psu_upgrade = set powershelf psu update -s {INDEX} -f {FILE}</t>
+-       rm_psu_upgrade = set powershelf psu update -s {INDEX} -f {FILE}</t>
         </is>
       </c>
       <c r="G26" s="84" t="b">
@@ -7499,7 +7500,7 @@
       <c r="E31" s="40" t="inlineStr">
         <is>
           <t>Two very different code paths: 
-- for prj_stage == "M5" it SFTP-uploads the three HWKEY .bin files to the BMC, then uses a shell command list over usb0 (10.235.100.0/31 point-to-point link) with scp -P 2200 to pull each key onto the GlacierPeak SoC and run cerberus_utility importsignedcert locally there — all three fuse commands (root CA idx 1, intermediate idx 2, device ID idx 0) run under a single rscm_lock.
+- for prj_stage == "M5" it SFTP-uploads the three HWKEY .bin files to the BMC, then uses a shell command list over usb0 (10.235.100.0/31 point-to-point link) with scp -P 2200 to pull each key onto the GlacierPeak SoC and run cerberus_utility importsignedcert locally there — all three fuse commands (root CA idx 1, intermediate idx 2, device ID idx 0) run under a single rm_lock.
 - For other stages it uses a raw pxssh session direct to the GlacierPeak SoC on port 8295 (user admin/admin), with up to 2 retries and a 90s backoff between attempts if the SoC is "busy". HWKey files are deleted from the BMC after fusing in both paths.</t>
         </is>
       </c>
@@ -7539,7 +7540,7 @@
           <t>- Security/identity-relevant, one-time step, M3-only. 
 - Unlike the Manticore/TIP flow this checks each slot independently — a partially-provisioned board (e.g. slot0 done, slot1 not) only provisions the missing slot. 
 - No verification of the -setCertificate output content is performed. 
-- Uses self.rscm_lock("RSCM", ...) around the actual burn to avoid concurrent RSCM access from other test threads.
+- Uses self.rm_lock("RM", ...) around the actual burn to avoid concurrent RM access from other test threads.
 - After both slots are set, it resets the FPGA and sleeps 300s before the final confirmation check.</t>
         </is>
       </c>
@@ -7844,7 +7845,7 @@
       </c>
       <c r="C41" s="43" t="inlineStr">
         <is>
-          <t>Check R-SCM FRU information</t>
+          <t>Check RM FRU information</t>
         </is>
       </c>
       <c r="D41" s="40" t="inlineStr">
@@ -7936,7 +7937,7 @@
       </c>
       <c r="C44" s="43" t="inlineStr">
         <is>
-          <t>Check System FRU via RSCM</t>
+          <t>Check System FRU via RM</t>
         </is>
       </c>
       <c r="D44" s="40" t="inlineStr">
@@ -7968,7 +7969,7 @@
       </c>
       <c r="C45" s="43" t="inlineStr">
         <is>
-          <t>Check DC-SCM(M1120) FRU via R-SCM</t>
+          <t>Check DC-SCM(M1120) FRU via RM</t>
         </is>
       </c>
       <c r="D45" s="40" t="inlineStr">
@@ -8004,7 +8005,7 @@
       </c>
       <c r="C46" s="43" t="inlineStr">
         <is>
-          <t>Check GlacierPeak FRU via R-SCM</t>
+          <t>Check GlacierPeak FRU via RM</t>
         </is>
       </c>
       <c r="D46" s="40" t="inlineStr">
@@ -8103,7 +8104,7 @@
       </c>
       <c r="C49" s="43" t="inlineStr">
         <is>
-          <t>Validates RSCM rack-level power capping behavior, including: - DCMI-based static power limit control - PSU alert-triggered throttling (SM_ALERT)</t>
+          <t>Validates RM rack-level power capping behavior, including: - DCMI-based static power limit control - PSU alert-triggered throttling (SM_ALERT)</t>
         </is>
       </c>
       <c r="D49" s="40" t="inlineStr">
@@ -8768,13 +8769,13 @@
       </c>
       <c r="D64" s="40" t="inlineStr">
         <is>
-          <t>PASS if 5/5 pings succeed (or the RSCM-routed SSH connect succeeds).</t>
+          <t>PASS if 5/5 pings succeed (or the RM-routed SSH connect succeeds).</t>
         </is>
       </c>
       <c r="E64" s="40" t="inlineStr">
         <is>
           <t>M1/M3: via a direct ICMP ping
-M5: ping via an SSH-through-RSCM reachability check</t>
+M5: ping via an SSH-through-RM reachability check</t>
         </is>
       </c>
       <c r="F64" s="75" t="n"/>
@@ -9242,7 +9243,7 @@
       </c>
       <c r="C78" s="43" t="inlineStr">
         <is>
-          <t>Runs fpgadiagnostics -dumpHealth (via a stage-appropriate SSH route: direct M3, RSCM-jumper M3, or RSCM-serial-proxy M5) and parses per-subsystem [FPGA-XXX] health lines, with specific waivers for known FPGA-NETWORK and FPGA-CONFIG warnings, and a one-time auto-reboot self-heal if the PCIe link status reads "WARNING" while in App mode.</t>
+          <t>Runs fpgadiagnostics -dumpHealth (via a stage-appropriate SSH route: direct M3, RM-jumper M3, or RM-serial-proxy M5) and parses per-subsystem [FPGA-XXX] health lines, with specific waivers for known FPGA-NETWORK and FPGA-CONFIG warnings, and a one-time auto-reboot self-heal if the PCIe link status reads "WARNING" while in App mode.</t>
         </is>
       </c>
       <c r="D78" s="40" t="inlineStr">
@@ -9694,7 +9695,7 @@
       <c r="E90" s="40" t="n"/>
       <c r="F90" s="43" t="inlineStr">
         <is>
-          <t>[ Check powershelf firmware version ] show powershelf psu info -s {INDEX} Capability IC Device ID Manufacturer ID Manufacturer Model Manufacturer Revision Manufacturer Serial Completion Code - - - - - If mismatch - - - - - [ Upgrade Rack SCM firmware version ] C heck fw package exists in RSCM show manager tftp list Upload fw to Rack-SCM set manager tftp get -s {IP} -f {FILE} Fw Upgrade set manager cerberus cmd -c pcdupdate /usr/srvroot/shared/{FILE}</t>
+          <t>[ Check powershelf firmware version ] show powershelf psu info -s {INDEX} Capability IC Device ID Manufacturer ID Manufacturer Model Manufacturer Revision Manufacturer Serial Completion Code - - - - - If mismatch - - - - - [ Upgrade Rack SCM firmware version ] C heck fw package exists in RM show manager tftp list Upload fw to Rack-SCM set manager tftp get -s {IP} -f {FILE} Fw Upgrade set manager cerberus cmd -c pcdupdate /usr/srvroot/shared/{FILE}</t>
         </is>
       </c>
       <c r="G90" s="47" t="n"/>
@@ -9802,7 +9803,7 @@
       </c>
       <c r="F92" s="43" t="inlineStr">
         <is>
-          <t>[Check RSCM Cerberus Version] show manager cerberus version - - - - - If mismatch - - - - - [Upgrade RSCM Cerberus] set manager cerberus update -f {FILE} [Check RSCM Cerberus PCD ID] set manager cerberus cmd -c pcdid - - - - - If mismatch - - - - - [Upgrade RSCM Cerberus PCD ID] set manager cerberus cmd -c pcdupdate /usr/srvroot/shared/{FILE} [Check RSCM Cerberus PFM ID] show manager cerberus pfm id -p 1 -r 0 - - - - - If mismatch - - - - - [Upgrade RSCM Cerberus PFM ID] set manager cerberus pfm update -f {FILE} -p 1 [Get RSCM information FAIL] show manager version - - - - - If mismatch - - - - - [Upgrade RSCM information] set manager fwupdate -f {FILE} [Check RSCM CPLD version] show manager cpld version - - - - - If mismatch - - - - - [Upgrade RSCM CPLD version] set manager cpld update -f {FILE}</t>
+          <t>[Check RM Cerberus Version] show manager cerberus version - - - - - If mismatch - - - - - [Upgrade RM Cerberus] set manager cerberus update -f {FILE} [Check RM Cerberus PCD ID] set manager cerberus cmd -c pcdid - - - - - If mismatch - - - - - [Upgrade RM Cerberus PCD ID] set manager cerberus cmd -c pcdupdate /usr/srvroot/shared/{FILE} [Check RM Cerberus PFM ID] show manager cerberus pfm id -p 1 -r 0 - - - - - If mismatch - - - - - [Upgrade RM Cerberus PFM ID] set manager cerberus pfm update -f {FILE} -p 1 [Get RM information FAIL] show manager version - - - - - If mismatch - - - - - [Upgrade RM information] set manager fwupdate -f {FILE} [Check RM CPLD version] show manager cpld version - - - - - If mismatch - - - - - [Upgrade RM CPLD version] set manager cpld update -f {FILE}</t>
         </is>
       </c>
       <c r="G92" s="47" t="n"/>
@@ -9821,22 +9822,22 @@
       <c r="J92" s="41" t="n"/>
       <c r="K92" s="42" t="inlineStr">
         <is>
-          <t>Check RSCM Cerberus Version PASS. Exp:1.5.7.5 Get:1.5.7.5
-Check RSCM PCD Version ID PASS. SF:0x1 Get:0x1
-Check RSCM PCD Platform ID PASS. SF:M4011 Get:M4011
-Check RSCM PFM ID Version PASS. Exp:0x3DA Get:0x3da
-Check RSCM information PASS. Exp:1.31.6, get_rootfs:1.31.6, get_kernel:1.31.6, get_package:1.31.6, get_device_tree:1.31.6
-Check RSCM CPLD Version PASS. Exp:V3.5 Get:V3.5
-Get RSCM Manager Type PASS. GET : 3OU_POWER_SHELF; EXP : 3OU_POWER_SHELF
-Get RSCM Host Name PASS. GET : rscm-hs-sr2-m4010; EXP : rscm-hs-sr2-m4010
-Get RSCM Uboot Version PASS. GET : 2021.01; EXP : 2021.01
-Get RSCM NTP Server PASS. GET : 172.52.0.1; EXP : 172.52.0.1
-Check All RSCM Version PASS.</t>
+          <t>Check RM Cerberus Version PASS. Exp:1.5.7.5 Get:1.5.7.5
+Check RM PCD Version ID PASS. SF:0x1 Get:0x1
+Check RM PCD Platform ID PASS. SF:M4011 Get:M4011
+Check RM PFM ID Version PASS. Exp:0x3DA Get:0x3da
+Check RM information PASS. Exp:1.31.6, get_rootfs:1.31.6, get_kernel:1.31.6, get_package:1.31.6, get_device_tree:1.31.6
+Check RM CPLD Version PASS. Exp:V3.5 Get:V3.5
+Get RM Manager Type PASS. GET : 3OU_POWER_SHELF; EXP : 3OU_POWER_SHELF
+Get RM Host Name PASS. GET : rm-hs-sr2-m4010; EXP : rm-hs-sr2-m4010
+Get RM Uboot Version PASS. GET : 2021.01; EXP : 2021.01
+Get RM NTP Server PASS. GET : 172.52.0.1; EXP : 172.52.0.1
+Check All RM Version PASS.</t>
         </is>
       </c>
       <c r="L92" s="31" t="inlineStr">
         <is>
-          <t>Matches CRD: Cerberus 1.5.7.5, PFMID 0x3DA, PCD M4011/0x1, R-SCM 1.31.6, CPLD V3.5.</t>
+          <t>Matches CRD: Cerberus 1.5.7.5, PFMID 0x3DA, PCD M4011/0x1, RM 1.31.6, CPLD V3.5.</t>
         </is>
       </c>
       <c r="M92" s="18" t="n"/>
@@ -9879,7 +9880,7 @@
       </c>
       <c r="F93" s="43" t="inlineStr">
         <is>
-          <t>[ Get system info via R-SCM ] show system info -i { RM_PORT } Mac Address SerialNumber BiosVersion BMCVersion CpldVersion DCSCMCpldVersion Count TotalSystemMemoryGib - - - - - If mismatch - - - - - [ Upgrade system firmware version ] set system file put -i {PORT} -f {FILE} set system bios update -i {PORT} -f {FILE} set system bmc update -i {PORT} -f {FILE}</t>
+          <t>[ Get system info via RM ] show system info -i { RM_PORT } Mac Address SerialNumber BiosVersion BMCVersion CpldVersion DCSCMCpldVersion Count TotalSystemMemoryGib - - - - - If mismatch - - - - - [ Upgrade system firmware version ] set system file put -i {PORT} -f {FILE} set system bios update -i {PORT} -f {FILE} set system bmc update -i {PORT} -f {FILE}</t>
         </is>
       </c>
       <c r="G93" s="47" t="b">
@@ -9898,7 +9899,7 @@
 DCSCMCpldVersion         check PASS. Get:                 03.06.00, Exp:                 03.06.00
 Count                    check PASS. Get:                        2, Exp:                        2
 TotalSystemMemoryGib     check PASS. Get:                      512, Exp:                      512
-[PASS] Check system info via R-SCM PASS
+[PASS] Check system info via RM PASS
 </t>
         </is>
       </c>
@@ -9913,7 +9914,7 @@
 DCSCMCpldVersion         check PASS. Get:                 03.06.00, Exp:                 03.06.00
 Count                    check PASS. Get:                        2, Exp:                        2
 TotalSystemMemoryGib     check PASS. Get:                      512, Exp:                      512
-[PASS] Check system info via R-SCM PASS"</t>
+[PASS] Check system info via RM PASS"</t>
         </is>
       </c>
       <c r="L93" s="31" t="inlineStr">
@@ -10854,7 +10855,7 @@
       </c>
       <c r="E14" s="43" t="inlineStr">
         <is>
-          <t>Uses Context.save_boot_state()/gs_load_ctx() to track reboot_count across the AC cycle. On M5 stage, routes the AC command through RSCM SSH instead of direct BMC IPMI.</t>
+          <t>Uses Context.save_boot_state()/gs_load_ctx() to track reboot_count across the AC cycle. On M5 stage, routes the AC command through RM SSH instead of direct BMC IPMI.</t>
         </is>
       </c>
       <c r="F14" s="43" t="inlineStr">
@@ -12248,7 +12249,7 @@
       </c>
       <c r="F12" s="43" t="inlineStr">
         <is>
-          <t>[Check RSCM Cerberus Version] show manager cerberus version - - - - - If mismatch - - - - - [Upgrade RSCM Cerberus] set manager cerberus update -f {FILE} [Check RSCM Cerberus PCD ID] set manager cerberus cmd -c pcdid - - - - - If mismatch - - - - - [Upgrade RSCM Cerberus PCD ID] set manager cerberus cmd -c pcdupdate /usr/srvroot/shared/{FILE} [Check RSCM Cerberus PFM ID] show manager cerberus pfm id -p 1 -r 0 - - - - - If mismatch - - - - - [Upgrade RSCM Cerberus PFM ID] set manager cerberus pfm update -f {FILE} -p 1 [Get RSCM information FAIL] show manager version - - - - - If mismatch - - - - - [Upgrade RSCM information] set manager fwupdate -f {FILE} [Check RSCM CPLD version] show manager cpld version - - - - - If mismatch - - - - - [Upgrade RSCM CPLD version] set manager cpld update -f {FILE}</t>
+          <t>[Check RM Cerberus Version] show manager cerberus version - - - - - If mismatch - - - - - [Upgrade RM Cerberus] set manager cerberus update -f {FILE} [Check RM Cerberus PCD ID] set manager cerberus cmd -c pcdid - - - - - If mismatch - - - - - [Upgrade RM Cerberus PCD ID] set manager cerberus cmd -c pcdupdate /usr/srvroot/shared/{FILE} [Check RM Cerberus PFM ID] show manager cerberus pfm id -p 1 -r 0 - - - - - If mismatch - - - - - [Upgrade RM Cerberus PFM ID] set manager cerberus pfm update -f {FILE} -p 1 [Get RM information FAIL] show manager version - - - - - If mismatch - - - - - [Upgrade RM information] set manager fwupdate -f {FILE} [Check RM CPLD version] show manager cpld version - - - - - If mismatch - - - - - [Upgrade RM CPLD version] set manager cpld update -f {FILE}</t>
         </is>
       </c>
       <c r="G12" s="47" t="n"/>
@@ -12257,34 +12258,34 @@
       </c>
       <c r="I12" s="63" t="inlineStr">
         <is>
-          <t>No rscm powershelf master in LAB. Waive</t>
+          <t>No rm powershelf master in LAB. Waive</t>
         </is>
       </c>
       <c r="J12" s="48" t="n"/>
       <c r="K12" s="42" t="inlineStr">
         <is>
-          <t>Check RSCM Cerberus Version PASS. Exp:1.5.7.5 Get:1.5.7.5
-Check RSCM PCD Version ID PASS. SF:0x1 Get:0x1
-Check RSCM PCD Platform ID PASS. SF:M4011 Get:M4011
-Check RSCM PFM ID Version PASS. Exp:0x3DA Get:0x3da
-Check RSCM information PASS. Exp:1.31.6, get_rootfs:1.31.6, get_kernel:1.31.6, get_package:1.31.6, get_device_tree:1.31.6
-Check RSCM CPLD Version PASS. Exp:V3.5 Get:V3.5
-Get RSCM Manager Type PASS. GET : 3OU_POWER_SHELF; EXP : 3OU_POWER_SHELF
-Get RSCM Host Name PASS. GET : rscm-hs-sr2-m4010; EXP : rscm-hs-sr2-m4010
-Get RSCM Uboot Version PASS. GET : 2021.01; EXP : 2021.01
-Get RSCM NTP Server PASS. GET : 172.52.0.1; EXP : 172.52.0.1
-Check All RSCM Version PASS.</t>
+          <t>Check RM Cerberus Version PASS. Exp:1.5.7.5 Get:1.5.7.5
+Check RM PCD Version ID PASS. SF:0x1 Get:0x1
+Check RM PCD Platform ID PASS. SF:M4011 Get:M4011
+Check RM PFM ID Version PASS. Exp:0x3DA Get:0x3da
+Check RM information PASS. Exp:1.31.6, get_rootfs:1.31.6, get_kernel:1.31.6, get_package:1.31.6, get_device_tree:1.31.6
+Check RM CPLD Version PASS. Exp:V3.5 Get:V3.5
+Get RM Manager Type PASS. GET : 3OU_POWER_SHELF; EXP : 3OU_POWER_SHELF
+Get RM Host Name PASS. GET : rm-hs-sr2-m4010; EXP : rm-hs-sr2-m4010
+Get RM Uboot Version PASS. GET : 2021.01; EXP : 2021.01
+Get RM NTP Server PASS. GET : 172.52.0.1; EXP : 172.52.0.1
+Check All RM Version PASS.</t>
         </is>
       </c>
       <c r="L12" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">Matches CRD
-R-SCM Cerberus 1.5.7.5
-R-SCM Cerberus PCD Version ID 0x1
-R-SCM Cerberus PCD Platform ID M4011
-R-SCM PFMID value 0x3DA
-R-SCM Firmware 1.31.6
-R-SCM CPLD V3.5
+RM Cerberus 1.5.7.5
+RM Cerberus PCD Version ID 0x1
+RM Cerberus PCD Platform ID M4011
+RM PFMID value 0x3DA
+RM Firmware 1.31.6
+RM CPLD V3.5
 </t>
         </is>
       </c>
@@ -12300,7 +12301,7 @@
       </c>
       <c r="C13" s="82" t="inlineStr">
         <is>
-          <t>Check the PSU firmware version on the power shelf via R-SCM for the current UUT. This function only performs the check on master nodes.</t>
+          <t>Check the PSU firmware version on the power shelf via RM for the current UUT. This function only performs the check on master nodes.</t>
         </is>
       </c>
       <c r="D13" s="82" t="inlineStr">
@@ -12309,7 +12310,7 @@
 - UUT is a master node.
 - All PSU serial numbers, manufacturers, and firmware versions match expected values.
 - Fail
-- Unable to get R-SCM IP.
+- Unable to get RM IP.
 - PSU information cannot be retrieved or parsed.
 - PSU not found in the expected list.
 - Firmware version mismatch and auto-upgrade fails.</t>
@@ -12357,7 +12358,7 @@
       </c>
       <c r="C14" s="82" t="inlineStr">
         <is>
-          <t>Check RSCM Health Status</t>
+          <t>Check RM Health Status</t>
         </is>
       </c>
       <c r="D14" s="82" t="inlineStr">
@@ -12395,7 +12396,7 @@
       <c r="C15" s="82" t="inlineStr">
         <is>
           <t>Check POWERSHELF Product Name
-Check RSCM Manager Type</t>
+Check RM Manager Type</t>
         </is>
       </c>
       <c r="D15" s="82" t="n"/>
@@ -12427,12 +12428,12 @@
       </c>
       <c r="C16" s="43" t="inlineStr">
         <is>
-          <t>C hecks UUT system information via the R-SCM interface and compares it with the expected configuration values .</t>
+          <t>C hecks UUT system information via the RM interface and compares it with the expected configuration values .</t>
         </is>
       </c>
       <c r="D16" s="43" t="inlineStr">
         <is>
-          <t>Pass All fields (MAC, SN, BIOS version, BMC version, CPLD versions, CPU count, and memory size) match expected values. Or mismatched fields are successfully auto-updated (if allowed). Fail Unable to retrieve system info from R-SCM. Mismatched field(s) and auto-upgrade is either disabled or unsuccessful.</t>
+          <t>Pass All fields (MAC, SN, BIOS version, BMC version, CPLD versions, CPU count, and memory size) match expected values. Or mismatched fields are successfully auto-updated (if allowed). Fail Unable to retrieve system info from RM. Mismatched field(s) and auto-upgrade is either disabled or unsuccessful.</t>
         </is>
       </c>
       <c r="E16" s="43" t="inlineStr">
@@ -12442,7 +12443,7 @@
       </c>
       <c r="F16" s="43" t="inlineStr">
         <is>
-          <t>[ Get system info via R-SCM ] show system info -i { RM_PORT } Mac Address SerialNumber BiosVersion BMCVersion CpldVersion DCSCMCpldVersion Count TotalSystemMemoryGib - - - - - If mismatch - - - - - [ Upgrade system firmware version ] set system file put -i {PORT} -f {FILE} set system bios update -i {PORT} -f {FILE} set system bmc update -i {PORT} -f {FILE}</t>
+          <t>[ Get system info via RM ] show system info -i { RM_PORT } Mac Address SerialNumber BiosVersion BMCVersion CpldVersion DCSCMCpldVersion Count TotalSystemMemoryGib - - - - - If mismatch - - - - - [ Upgrade system firmware version ] set system file put -i {PORT} -f {FILE} set system bios update -i {PORT} -f {FILE} set system bmc update -i {PORT} -f {FILE}</t>
         </is>
       </c>
       <c r="G16" s="47" t="b">
@@ -12463,7 +12464,7 @@
 DCSCMCpldVersion         check PASS. Get:                 03.06.00, Exp:                 03.06.00
 Count                    check PASS. Get:                        2, Exp:                        2
 TotalSystemMemoryGib     check PASS. Get:                      512, Exp:                      512
-[PASS] Check system info via R-SCM PASS"</t>
+[PASS] Check system info via RM PASS"</t>
         </is>
       </c>
       <c r="L16" s="31" t="inlineStr">
@@ -12484,7 +12485,7 @@
       </c>
       <c r="C17" s="43" t="inlineStr">
         <is>
-          <t>Check R-SCM FRU information</t>
+          <t>Check RM FRU information</t>
         </is>
       </c>
       <c r="D17" s="43" t="inlineStr">
@@ -12573,7 +12574,7 @@
       </c>
       <c r="C20" s="43" t="inlineStr">
         <is>
-          <t>Check System FRU via RSCM</t>
+          <t>Check System FRU via RM</t>
         </is>
       </c>
       <c r="D20" s="43" t="inlineStr">
@@ -12604,7 +12605,7 @@
       </c>
       <c r="C21" s="43" t="inlineStr">
         <is>
-          <t>Check DC-SCM(M1120) FRU via R-SCM</t>
+          <t>Check DC-SCM(M1120) FRU via RM</t>
         </is>
       </c>
       <c r="D21" s="43" t="inlineStr">
@@ -12639,7 +12640,7 @@
       </c>
       <c r="C22" s="43" t="inlineStr">
         <is>
-          <t>Check GlacierPeak FRU via R-SCM</t>
+          <t>Check GlacierPeak FRU via RM</t>
         </is>
       </c>
       <c r="D22" s="43" t="inlineStr">
@@ -13476,13 +13477,13 @@
       </c>
       <c r="D42" s="43" t="inlineStr">
         <is>
-          <t>PASS if 5/5 pings succeed (or the RSCM-routed SSH connect succeeds).</t>
+          <t>PASS if 5/5 pings succeed (or the RM-routed SSH connect succeeds).</t>
         </is>
       </c>
       <c r="E42" s="43" t="inlineStr">
         <is>
           <t>M1/M3: via a direct ICMP ping
-M5: ping via an SSH-through-RSCM reachability check</t>
+M5: ping via an SSH-through-RM reachability check</t>
         </is>
       </c>
       <c r="F42" s="43" t="n"/>
@@ -14082,7 +14083,7 @@
       </c>
       <c r="C60" s="43" t="inlineStr">
         <is>
-          <t>Runs fpgadiagnostics -dumpHealth (via a stage-appropriate SSH route: direct M3, RSCM-jumper M3, or RSCM-serial-proxy M5) and parses per-subsystem [FPGA-XXX] health lines, with specific waivers for known FPGA-NETWORK and FPGA-CONFIG warnings, and a one-time auto-reboot self-heal if the PCIe link status reads "WARNING" while in App mode.</t>
+          <t>Runs fpgadiagnostics -dumpHealth (via a stage-appropriate SSH route: direct M3, RM-jumper M3, or RM-serial-proxy M5) and parses per-subsystem [FPGA-XXX] health lines, with specific waivers for known FPGA-NETWORK and FPGA-CONFIG warnings, and a one-time auto-reboot self-heal if the PCIe link status reads "WARNING" while in App mode.</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
@@ -14162,7 +14163,7 @@
       </c>
       <c r="E62" s="43" t="inlineStr">
         <is>
-          <t>Multi-stage, stateful check keyed on the presence of /vol/data/persistent/tests/golden_status.txt on the BMC. If the log doesn't exist yet, the function uploads SoCFPGAGoldenTestSvc.service and fpga_golden_check.py to the BMC, switches GP into golden boot mode (cerberus_utility fpgasetbootmode 0), forces an AC cycle (RSCM rscm_system_ac on M5, gs_pdb_ac_cycle otherwise) to make the mode take effect, and then returns 1 — meaning the first pass of this item after an image/config change always intentionally fails and needs a subsequent PRETEST re-run to actually validate the version. On version mismatch with fpga_gp_fw_upgrade TRUE, it calls _gp_fpga_softnic_upgrade() and then re-generates the golden log (also returning 1) rather than re-checking in the same pass.</t>
+          <t>Multi-stage, stateful check keyed on the presence of /vol/data/persistent/tests/golden_status.txt on the BMC. If the log doesn't exist yet, the function uploads SoCFPGAGoldenTestSvc.service and fpga_golden_check.py to the BMC, switches GP into golden boot mode (cerberus_utility fpgasetbootmode 0), forces an AC cycle (RM rm_system_ac on M5, gs_pdb_ac_cycle otherwise) to make the mode take effect, and then returns 1 — meaning the first pass of this item after an image/config change always intentionally fails and needs a subsequent PRETEST re-run to actually validate the version. On version mismatch with fpga_gp_fw_upgrade TRUE, it calls _gp_fpga_softnic_upgrade() and then re-generates the golden log (also returning 1) rather than re-checking in the same pass.</t>
         </is>
       </c>
       <c r="F62" s="43" t="n"/>
@@ -14198,7 +14199,7 @@
       <c r="E63" s="43" t="inlineStr">
         <is>
           <t>Two very different code paths: 
-- for prj_stage == "M5" it SFTP-uploads the three HWKEY .bin files to the BMC, then uses a shell command list over usb0 (10.235.100.0/31 point-to-point link) with scp -P 2200 to pull each key onto the GlacierPeak SoC and run cerberus_utility importsignedcert locally there — all three fuse commands (root CA idx 1, intermediate idx 2, device ID idx 0) run under a single rscm_lock.
+- for prj_stage == "M5" it SFTP-uploads the three HWKEY .bin files to the BMC, then uses a shell command list over usb0 (10.235.100.0/31 point-to-point link) with scp -P 2200 to pull each key onto the GlacierPeak SoC and run cerberus_utility importsignedcert locally there — all three fuse commands (root CA idx 1, intermediate idx 2, device ID idx 0) run under a single rm_lock.
 - For other stages it uses a raw pxssh session direct to the GlacierPeak SoC on port 8295 (user admin/admin), with up to 2 retries and a 90s backoff between attempts if the SoC is "busy". HWKey files are deleted from the BMC after fusing in both paths.</t>
         </is>
       </c>
@@ -14237,7 +14238,7 @@
           <t>- Security/identity-relevant, one-time step, M3-only. 
 - Unlike the Manticore/TIP flow this checks each slot independently — a partially-provisioned board (e.g. slot0 done, slot1 not) only provisions the missing slot. 
 - No verification of the -setCertificate output content is performed. 
-- Uses self.rscm_lock("RSCM", ...) around the actual burn to avoid concurrent RSCM access from other test threads.
+- Uses self.rm_lock("RM", ...) around the actual burn to avoid concurrent RM access from other test threads.
 - After both slots are set, it resets the FPGA and sleeps 300s before the final confirmation check.</t>
         </is>
       </c>

</xml_diff>